<commit_message>
organizing data repo for publication (1st)
</commit_message>
<xml_diff>
--- a/data/hyporheic_fluxes/trapGSD_hypflux_organized.xlsx
+++ b/data/hyporheic_fluxes/trapGSD_hypflux_organized.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\sediment_trap_paper\data\hyporheic_fluxes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93F218C-B604-4FF8-8D04-7615501F17C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{475F06C0-3AE8-4E67-BCE0-B1F470DA10B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{8606DF0C-3933-40BB-BE19-03FC0B44297F}"/>
+    <workbookView xWindow="-25320" yWindow="360" windowWidth="25440" windowHeight="15270" activeTab="2" xr2:uid="{8606DF0C-3933-40BB-BE19-03FC0B44297F}"/>
   </bookViews>
   <sheets>
     <sheet name="Spring Weights" sheetId="1" r:id="rId1"/>
@@ -2921,32 +2921,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="29" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="31" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2957,25 +2957,31 @@
     <xf numFmtId="0" fontId="0" fillId="31" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="38" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="29" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3014,41 +3020,50 @@
     <xf numFmtId="0" fontId="0" fillId="36" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="31" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="38" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="28" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="29" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="30" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3059,28 +3074,13 @@
     <xf numFmtId="0" fontId="0" fillId="30" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4703,7 +4703,7 @@
                   <c:v>0.42806196398944324</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.43334548628417668</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>-0.26191713426081537</c:v>
@@ -8706,7 +8706,7 @@
                   <c:v>1.5015923261390882</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.4248532844281436</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0.6861382550335573</c:v>
@@ -8748,10 +8748,10 @@
                   <c:v>5.7776999999999994</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7.0016999999999996</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>11.661999999999999</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>10.2044</c:v>
@@ -8883,7 +8883,7 @@
                   <c:v>1.3819777993151134</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.71701174606419926</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>1.5524268675721558</c:v>
@@ -9054,7 +9054,7 @@
                   <c:v>1.5015923261390882</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.4248532844281436</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0.6861382550335573</c:v>
@@ -9090,7 +9090,7 @@
                   <c:v>1.3819777993151134</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.71701174606419926</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>1.5524268675721558</c:v>
@@ -9129,10 +9129,10 @@
                   <c:v>5.7776999999999994</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7.0016999999999996</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>11.661999999999999</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>10.2044</c:v>
@@ -9660,10 +9660,10 @@
                   <c:v>8.0606000000000009</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.8309999999999995</c:v>
+                  <c:v>15.135</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-14.6675</c:v>
+                  <c:v>4.6359000000000004</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>-5.1329000000000011</c:v>
@@ -9699,10 +9699,10 @@
                   <c:v>9.0438957452519855</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5.1789754851130283</c:v>
+                  <c:v>17.130122200684887</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>18.099126508969356</c:v>
+                  <c:v>-5.6020617449664432</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>-6.0971413133504697</c:v>
@@ -10024,10 +10024,10 @@
                   <c:v>4.6365499999999997</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.8309999999999995</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>14.6675</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>-5.3126999999999995</c:v>
@@ -10054,10 +10054,10 @@
                   <c:v>5.1529157327069051</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5.1789754851130283</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18.099126508969356</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>-5.7985584551809488</c:v>
@@ -10509,7 +10509,7 @@
                   <c:v>0.82482620575765719</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.43334548628417668</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>-0.25314346921600916</c:v>
@@ -20564,22 +20564,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:40" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="AG1" s="481" t="s">
+      <c r="AG1" s="508" t="s">
         <v>122</v>
       </c>
-      <c r="AH1" s="481" t="s">
+      <c r="AH1" s="508" t="s">
         <v>57</v>
       </c>
-      <c r="AI1" s="481" t="s">
+      <c r="AI1" s="508" t="s">
         <v>52</v>
       </c>
-      <c r="AJ1" s="481" t="s">
+      <c r="AJ1" s="508" t="s">
         <v>121</v>
       </c>
-      <c r="AK1" s="475" t="s">
+      <c r="AK1" s="518" t="s">
         <v>57</v>
       </c>
-      <c r="AL1" s="475" t="s">
+      <c r="AL1" s="518" t="s">
         <v>52</v>
       </c>
     </row>
@@ -20656,23 +20656,23 @@
       <c r="Y2" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="AB2" s="478" t="s">
+      <c r="AB2" s="515" t="s">
         <v>25</v>
       </c>
-      <c r="AC2" s="479"/>
-      <c r="AD2" s="482" t="s">
+      <c r="AC2" s="521"/>
+      <c r="AD2" s="475" t="s">
         <v>58</v>
       </c>
-      <c r="AE2" s="482"/>
+      <c r="AE2" s="475"/>
       <c r="AF2" s="97" t="s">
         <v>97</v>
       </c>
-      <c r="AG2" s="483"/>
-      <c r="AH2" s="481"/>
-      <c r="AI2" s="481"/>
-      <c r="AJ2" s="481"/>
-      <c r="AK2" s="475"/>
-      <c r="AL2" s="475"/>
+      <c r="AG2" s="522"/>
+      <c r="AH2" s="508"/>
+      <c r="AI2" s="508"/>
+      <c r="AJ2" s="508"/>
+      <c r="AK2" s="518"/>
+      <c r="AL2" s="518"/>
     </row>
     <row r="3" spans="2:40" x14ac:dyDescent="0.25">
       <c r="B3" s="14">
@@ -20901,8 +20901,8 @@
         <v>4.4862982062414796</v>
       </c>
       <c r="AM4" s="395">
-        <f>SUM(AG4:AI4)</f>
-        <v>3.5666000000000149</v>
+        <f>SUM(AG4:AI4)+AD4</f>
+        <v>33.736500000000014</v>
       </c>
       <c r="AN4" s="395" cm="1">
         <f t="array" ref="AN4">SUM(AD4:AE4+AH4:AI4)</f>
@@ -21028,8 +21028,8 @@
         <v>4.6747701009495621</v>
       </c>
       <c r="AM5" s="395">
-        <f t="shared" ref="AM5:AM15" si="4">SUM(AG5:AI5)</f>
-        <v>2.7728000000000042</v>
+        <f t="shared" ref="AM5:AM15" si="4">SUM(AG5:AI5)+AD5</f>
+        <v>16.421100000000006</v>
       </c>
       <c r="AN5" s="395" cm="1">
         <f t="array" ref="AN5">SUM(AD5:AE5+AH5:AI5)</f>
@@ -21156,7 +21156,7 @@
       </c>
       <c r="AM6" s="395">
         <f t="shared" si="4"/>
-        <v>2.9189000000000047</v>
+        <v>32.998700000000007</v>
       </c>
       <c r="AN6" s="395" cm="1">
         <f t="array" ref="AN6">SUM(AD6:AE6+AH6:AI6)</f>
@@ -21283,7 +21283,7 @@
       </c>
       <c r="AM7" s="395">
         <f t="shared" si="4"/>
-        <v>2.5218999999999983</v>
+        <v>29.533599999999996</v>
       </c>
       <c r="AN7" s="395" cm="1">
         <f t="array" ref="AN7">SUM(AD7:AE7+AH7:AI7)</f>
@@ -21410,7 +21410,7 @@
       </c>
       <c r="AM8" s="395">
         <f t="shared" si="4"/>
-        <v>6.1195000000000022</v>
+        <v>38.480800000000002</v>
       </c>
       <c r="AN8" s="395" cm="1">
         <f t="array" ref="AN8">SUM(AD8:AE8+AH8:AI8)</f>
@@ -21537,7 +21537,7 @@
       </c>
       <c r="AM9" s="395">
         <f t="shared" si="4"/>
-        <v>3.871399999999996</v>
+        <v>17.743799999999997</v>
       </c>
       <c r="AN9" s="395" cm="1">
         <f t="array" ref="AN9">SUM(AD9:AE9+AH9:AI9)</f>
@@ -21664,7 +21664,7 @@
       </c>
       <c r="AM10" s="395">
         <f t="shared" si="4"/>
-        <v>5.6356000000000046</v>
+        <v>49.202600000000004</v>
       </c>
       <c r="AN10" s="395" cm="1">
         <f t="array" ref="AN10">SUM(AD10:AE10+AH10:AI10)</f>
@@ -21791,7 +21791,7 @@
       </c>
       <c r="AM11" s="395">
         <f t="shared" si="4"/>
-        <v>2.2792999999999988</v>
+        <v>23.644499999999997</v>
       </c>
       <c r="AN11" s="395" cm="1">
         <f t="array" ref="AN11">SUM(AD11:AE11+AH11:AI11)</f>
@@ -21918,7 +21918,7 @@
       </c>
       <c r="AM12" s="395">
         <f t="shared" si="4"/>
-        <v>1.0524999999999998</v>
+        <v>17.332099999999997</v>
       </c>
       <c r="AN12" s="395" cm="1">
         <f t="array" ref="AN12">SUM(AD12:AE12+AH12:AI12)</f>
@@ -22045,7 +22045,7 @@
       </c>
       <c r="AM13" s="395">
         <f t="shared" si="4"/>
-        <v>1.5746000000000033</v>
+        <v>11.829200000000004</v>
       </c>
       <c r="AN13" s="395" cm="1">
         <f t="array" ref="AN13">SUM(AD13:AE13+AH13:AI13)</f>
@@ -22172,7 +22172,7 @@
       </c>
       <c r="AM14" s="395">
         <f t="shared" si="4"/>
-        <v>3.2265000000000064</v>
+        <v>16.687600000000007</v>
       </c>
       <c r="AN14" s="395" cm="1">
         <f t="array" ref="AN14">SUM(AD14:AE14+AH14:AI14)</f>
@@ -22299,7 +22299,7 @@
       </c>
       <c r="AM15" s="395">
         <f t="shared" si="4"/>
-        <v>2.4796999999999936</v>
+        <v>23.520599999999995</v>
       </c>
       <c r="AN15" s="395" cm="1">
         <f t="array" ref="AN15">SUM(AD15:AE15+AH15:AI15)</f>
@@ -22379,22 +22379,22 @@
       <c r="Y16" s="41">
         <v>1.1583636475738333</v>
       </c>
-      <c r="AG16" s="481" t="s">
+      <c r="AG16" s="508" t="s">
         <v>122</v>
       </c>
-      <c r="AH16" s="481" t="s">
+      <c r="AH16" s="508" t="s">
         <v>57</v>
       </c>
-      <c r="AI16" s="481" t="s">
+      <c r="AI16" s="508" t="s">
         <v>52</v>
       </c>
-      <c r="AJ16" s="481" t="s">
+      <c r="AJ16" s="508" t="s">
         <v>56</v>
       </c>
-      <c r="AK16" s="475" t="s">
+      <c r="AK16" s="518" t="s">
         <v>57</v>
       </c>
-      <c r="AL16" s="475" t="s">
+      <c r="AL16" s="518" t="s">
         <v>52</v>
       </c>
       <c r="AN16" s="395"/>
@@ -22473,23 +22473,23 @@
         <v>1.2284974412725813</v>
       </c>
       <c r="Z17" s="395"/>
-      <c r="AB17" s="478" t="s">
+      <c r="AB17" s="515" t="s">
         <v>40</v>
       </c>
-      <c r="AC17" s="480"/>
-      <c r="AD17" s="482" t="s">
+      <c r="AC17" s="516"/>
+      <c r="AD17" s="475" t="s">
         <v>58</v>
       </c>
-      <c r="AE17" s="482"/>
+      <c r="AE17" s="475"/>
       <c r="AF17" s="97" t="s">
         <v>97</v>
       </c>
-      <c r="AG17" s="483"/>
-      <c r="AH17" s="481"/>
-      <c r="AI17" s="481"/>
-      <c r="AJ17" s="481"/>
-      <c r="AK17" s="475"/>
-      <c r="AL17" s="475"/>
+      <c r="AG17" s="522"/>
+      <c r="AH17" s="508"/>
+      <c r="AI17" s="508"/>
+      <c r="AJ17" s="508"/>
+      <c r="AK17" s="518"/>
+      <c r="AL17" s="518"/>
       <c r="AN17" s="395"/>
     </row>
     <row r="18" spans="2:40" x14ac:dyDescent="0.25">
@@ -24176,14 +24176,14 @@
       <c r="Y32" s="41">
         <v>6.9971946482520506</v>
       </c>
-      <c r="AA32" s="476" t="s">
+      <c r="AA32" s="519" t="s">
         <v>25</v>
       </c>
-      <c r="AB32" s="476"/>
-      <c r="AC32" s="477" t="s">
+      <c r="AB32" s="519"/>
+      <c r="AC32" s="520" t="s">
         <v>40</v>
       </c>
-      <c r="AD32" s="477"/>
+      <c r="AD32" s="520"/>
       <c r="AI32" s="229" t="s">
         <v>73</v>
       </c>
@@ -25760,10 +25760,10 @@
       </c>
     </row>
     <row r="49" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="AB49" s="482" t="s">
+      <c r="AB49" s="475" t="s">
         <v>132</v>
       </c>
-      <c r="AC49" s="482"/>
+      <c r="AC49" s="475"/>
       <c r="AJ49" s="232" t="s">
         <v>79</v>
       </c>
@@ -25988,34 +25988,34 @@
       </c>
     </row>
     <row r="55" spans="2:39" x14ac:dyDescent="0.25">
-      <c r="B55" s="490" t="s">
+      <c r="B55" s="512" t="s">
         <v>1</v>
       </c>
-      <c r="C55" s="491"/>
-      <c r="D55" s="491"/>
-      <c r="E55" s="491"/>
-      <c r="F55" s="492"/>
-      <c r="G55" s="490" t="s">
+      <c r="C55" s="513"/>
+      <c r="D55" s="513"/>
+      <c r="E55" s="513"/>
+      <c r="F55" s="514"/>
+      <c r="G55" s="512" t="s">
         <v>2</v>
       </c>
-      <c r="H55" s="491"/>
-      <c r="I55" s="491"/>
-      <c r="J55" s="491"/>
-      <c r="K55" s="492"/>
-      <c r="L55" s="490" t="s">
+      <c r="H55" s="513"/>
+      <c r="I55" s="513"/>
+      <c r="J55" s="513"/>
+      <c r="K55" s="514"/>
+      <c r="L55" s="512" t="s">
         <v>3</v>
       </c>
-      <c r="M55" s="491"/>
-      <c r="N55" s="491"/>
-      <c r="O55" s="491"/>
-      <c r="P55" s="492"/>
-      <c r="Q55" s="490" t="s">
+      <c r="M55" s="513"/>
+      <c r="N55" s="513"/>
+      <c r="O55" s="513"/>
+      <c r="P55" s="514"/>
+      <c r="Q55" s="512" t="s">
         <v>4</v>
       </c>
-      <c r="R55" s="491"/>
-      <c r="S55" s="491"/>
-      <c r="T55" s="491"/>
-      <c r="U55" s="492"/>
+      <c r="R55" s="513"/>
+      <c r="S55" s="513"/>
+      <c r="T55" s="513"/>
+      <c r="U55" s="514"/>
       <c r="AA55" s="67" t="s">
         <v>110</v>
       </c>
@@ -26028,7 +26028,7 @@
         <v>49.763951397452743</v>
       </c>
       <c r="AD55" s="85">
-        <f t="shared" si="19"/>
+        <f>SUM(AE55:AH55)</f>
         <v>49.763951397452736</v>
       </c>
       <c r="AE55" s="85">
@@ -26317,17 +26317,17 @@
       <c r="U58" s="169">
         <v>56.48097393940624</v>
       </c>
-      <c r="AB58" s="478" t="s">
+      <c r="AB58" s="515" t="s">
         <v>135</v>
       </c>
-      <c r="AC58" s="480"/>
-      <c r="AI58" s="493" t="s">
+      <c r="AC58" s="516"/>
+      <c r="AI58" s="517" t="s">
         <v>136</v>
       </c>
-      <c r="AJ58" s="493"/>
-      <c r="AK58" s="493"/>
-      <c r="AL58" s="493"/>
-      <c r="AM58" s="493"/>
+      <c r="AJ58" s="517"/>
+      <c r="AK58" s="517"/>
+      <c r="AL58" s="517"/>
+      <c r="AM58" s="517"/>
     </row>
     <row r="59" spans="2:39" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B59" s="170">
@@ -27353,10 +27353,10 @@
     </row>
     <row r="69" spans="2:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="AA69" s="215"/>
-      <c r="AB69" s="482" t="s">
+      <c r="AB69" s="475" t="s">
         <v>132</v>
       </c>
-      <c r="AC69" s="482"/>
+      <c r="AC69" s="475"/>
     </row>
     <row r="70" spans="2:40" x14ac:dyDescent="0.25">
       <c r="B70" s="484" t="s">
@@ -27554,7 +27554,7 @@
         <v>-17.267499999999998</v>
       </c>
       <c r="AK73" s="85">
-        <f t="shared" si="38"/>
+        <f>AC60-AC51</f>
         <v>-16.659925266373641</v>
       </c>
       <c r="AM73">
@@ -27853,10 +27853,10 @@
         <v>0.97190567716775433</v>
       </c>
       <c r="AA78" s="474"/>
-      <c r="AB78" s="478" t="s">
+      <c r="AB78" s="515" t="s">
         <v>135</v>
       </c>
-      <c r="AC78" s="480"/>
+      <c r="AC78" s="516"/>
       <c r="AI78" s="69" t="s">
         <v>111</v>
       </c>
@@ -28154,20 +28154,20 @@
       </c>
     </row>
     <row r="85" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="B85" s="487" t="s">
+      <c r="B85" s="509" t="s">
         <v>7</v>
       </c>
-      <c r="C85" s="488"/>
-      <c r="D85" s="488"/>
-      <c r="E85" s="488"/>
-      <c r="F85" s="489"/>
-      <c r="G85" s="487" t="s">
+      <c r="C85" s="510"/>
+      <c r="D85" s="510"/>
+      <c r="E85" s="510"/>
+      <c r="F85" s="511"/>
+      <c r="G85" s="509" t="s">
         <v>8</v>
       </c>
-      <c r="H85" s="488"/>
-      <c r="I85" s="488"/>
-      <c r="J85" s="488"/>
-      <c r="K85" s="489"/>
+      <c r="H85" s="510"/>
+      <c r="I85" s="510"/>
+      <c r="J85" s="510"/>
+      <c r="K85" s="511"/>
       <c r="M85" t="s">
         <v>119</v>
       </c>
@@ -28663,34 +28663,34 @@
     </row>
     <row r="99" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="100" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B100" s="494" t="s">
+      <c r="B100" s="496" t="s">
         <v>9</v>
       </c>
-      <c r="C100" s="495"/>
-      <c r="D100" s="495"/>
-      <c r="E100" s="495"/>
-      <c r="F100" s="496"/>
-      <c r="G100" s="494" t="s">
+      <c r="C100" s="497"/>
+      <c r="D100" s="497"/>
+      <c r="E100" s="497"/>
+      <c r="F100" s="498"/>
+      <c r="G100" s="496" t="s">
         <v>10</v>
       </c>
-      <c r="H100" s="495"/>
-      <c r="I100" s="495"/>
-      <c r="J100" s="495"/>
-      <c r="K100" s="496"/>
-      <c r="L100" s="497" t="s">
+      <c r="H100" s="497"/>
+      <c r="I100" s="497"/>
+      <c r="J100" s="497"/>
+      <c r="K100" s="498"/>
+      <c r="L100" s="499" t="s">
         <v>11</v>
       </c>
-      <c r="M100" s="498"/>
-      <c r="N100" s="498"/>
-      <c r="O100" s="498"/>
-      <c r="P100" s="499"/>
-      <c r="Q100" s="494" t="s">
+      <c r="M100" s="500"/>
+      <c r="N100" s="500"/>
+      <c r="O100" s="500"/>
+      <c r="P100" s="501"/>
+      <c r="Q100" s="496" t="s">
         <v>12</v>
       </c>
-      <c r="R100" s="495"/>
-      <c r="S100" s="495"/>
-      <c r="T100" s="495"/>
-      <c r="U100" s="496"/>
+      <c r="R100" s="497"/>
+      <c r="S100" s="497"/>
+      <c r="T100" s="497"/>
+      <c r="U100" s="498"/>
     </row>
     <row r="101" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B101" s="183" t="s">
@@ -29512,34 +29512,34 @@
     </row>
     <row r="114" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="115" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B115" s="500" t="s">
+      <c r="B115" s="502" t="s">
         <v>13</v>
       </c>
-      <c r="C115" s="501"/>
-      <c r="D115" s="501"/>
-      <c r="E115" s="501"/>
-      <c r="F115" s="502"/>
-      <c r="G115" s="500" t="s">
+      <c r="C115" s="503"/>
+      <c r="D115" s="503"/>
+      <c r="E115" s="503"/>
+      <c r="F115" s="504"/>
+      <c r="G115" s="502" t="s">
         <v>14</v>
       </c>
-      <c r="H115" s="501"/>
-      <c r="I115" s="501"/>
-      <c r="J115" s="501"/>
-      <c r="K115" s="502"/>
-      <c r="L115" s="503" t="s">
+      <c r="H115" s="503"/>
+      <c r="I115" s="503"/>
+      <c r="J115" s="503"/>
+      <c r="K115" s="504"/>
+      <c r="L115" s="505" t="s">
         <v>15</v>
       </c>
-      <c r="M115" s="504"/>
-      <c r="N115" s="504"/>
-      <c r="O115" s="504"/>
-      <c r="P115" s="505"/>
-      <c r="Q115" s="500" t="s">
+      <c r="M115" s="506"/>
+      <c r="N115" s="506"/>
+      <c r="O115" s="506"/>
+      <c r="P115" s="507"/>
+      <c r="Q115" s="502" t="s">
         <v>16</v>
       </c>
-      <c r="R115" s="501"/>
-      <c r="S115" s="501"/>
-      <c r="T115" s="501"/>
-      <c r="U115" s="502"/>
+      <c r="R115" s="503"/>
+      <c r="S115" s="503"/>
+      <c r="T115" s="503"/>
+      <c r="U115" s="504"/>
     </row>
     <row r="116" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B116" s="193" t="s">
@@ -30375,13 +30375,13 @@
       <c r="I130" s="485"/>
       <c r="J130" s="485"/>
       <c r="K130" s="486"/>
-      <c r="L130" s="506" t="s">
+      <c r="L130" s="487" t="s">
         <v>19</v>
       </c>
-      <c r="M130" s="507"/>
-      <c r="N130" s="507"/>
-      <c r="O130" s="507"/>
-      <c r="P130" s="508"/>
+      <c r="M130" s="488"/>
+      <c r="N130" s="488"/>
+      <c r="O130" s="488"/>
+      <c r="P130" s="489"/>
       <c r="Q130" s="484" t="s">
         <v>20</v>
       </c>
@@ -31210,27 +31210,27 @@
     </row>
     <row r="144" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="145" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B145" s="509" t="s">
+      <c r="B145" s="490" t="s">
         <v>21</v>
       </c>
-      <c r="C145" s="510"/>
-      <c r="D145" s="510"/>
-      <c r="E145" s="510"/>
-      <c r="F145" s="511"/>
-      <c r="G145" s="509" t="s">
+      <c r="C145" s="491"/>
+      <c r="D145" s="491"/>
+      <c r="E145" s="491"/>
+      <c r="F145" s="492"/>
+      <c r="G145" s="490" t="s">
         <v>22</v>
       </c>
-      <c r="H145" s="510"/>
-      <c r="I145" s="510"/>
-      <c r="J145" s="510"/>
-      <c r="K145" s="511"/>
-      <c r="L145" s="512" t="s">
+      <c r="H145" s="491"/>
+      <c r="I145" s="491"/>
+      <c r="J145" s="491"/>
+      <c r="K145" s="492"/>
+      <c r="L145" s="493" t="s">
         <v>23</v>
       </c>
-      <c r="M145" s="513"/>
-      <c r="N145" s="513"/>
-      <c r="O145" s="513"/>
-      <c r="P145" s="514"/>
+      <c r="M145" s="494"/>
+      <c r="N145" s="494"/>
+      <c r="O145" s="494"/>
+      <c r="P145" s="495"/>
     </row>
     <row r="146" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B146" s="203" t="s">
@@ -31856,36 +31856,6 @@
     </row>
   </sheetData>
   <mergeCells count="46">
-    <mergeCell ref="B130:F130"/>
-    <mergeCell ref="G130:K130"/>
-    <mergeCell ref="L130:P130"/>
-    <mergeCell ref="Q130:U130"/>
-    <mergeCell ref="B145:F145"/>
-    <mergeCell ref="G145:K145"/>
-    <mergeCell ref="L145:P145"/>
-    <mergeCell ref="B100:F100"/>
-    <mergeCell ref="G100:K100"/>
-    <mergeCell ref="L100:P100"/>
-    <mergeCell ref="Q100:U100"/>
-    <mergeCell ref="B115:F115"/>
-    <mergeCell ref="G115:K115"/>
-    <mergeCell ref="L115:P115"/>
-    <mergeCell ref="Q115:U115"/>
-    <mergeCell ref="AH16:AH17"/>
-    <mergeCell ref="AI16:AI17"/>
-    <mergeCell ref="B70:F70"/>
-    <mergeCell ref="G70:K70"/>
-    <mergeCell ref="B85:F85"/>
-    <mergeCell ref="G85:K85"/>
-    <mergeCell ref="B55:F55"/>
-    <mergeCell ref="G55:K55"/>
-    <mergeCell ref="L55:P55"/>
-    <mergeCell ref="Q55:U55"/>
-    <mergeCell ref="AB49:AC49"/>
-    <mergeCell ref="AB58:AC58"/>
-    <mergeCell ref="AI58:AM58"/>
-    <mergeCell ref="AB69:AC69"/>
-    <mergeCell ref="AB78:AC78"/>
     <mergeCell ref="AL1:AL2"/>
     <mergeCell ref="AL16:AL17"/>
     <mergeCell ref="AK16:AK17"/>
@@ -31902,6 +31872,36 @@
     <mergeCell ref="AH1:AH2"/>
     <mergeCell ref="AI1:AI2"/>
     <mergeCell ref="AG16:AG17"/>
+    <mergeCell ref="AH16:AH17"/>
+    <mergeCell ref="AI16:AI17"/>
+    <mergeCell ref="B70:F70"/>
+    <mergeCell ref="G70:K70"/>
+    <mergeCell ref="B85:F85"/>
+    <mergeCell ref="G85:K85"/>
+    <mergeCell ref="B55:F55"/>
+    <mergeCell ref="G55:K55"/>
+    <mergeCell ref="L55:P55"/>
+    <mergeCell ref="Q55:U55"/>
+    <mergeCell ref="AB49:AC49"/>
+    <mergeCell ref="AB58:AC58"/>
+    <mergeCell ref="AI58:AM58"/>
+    <mergeCell ref="AB69:AC69"/>
+    <mergeCell ref="AB78:AC78"/>
+    <mergeCell ref="B100:F100"/>
+    <mergeCell ref="G100:K100"/>
+    <mergeCell ref="L100:P100"/>
+    <mergeCell ref="Q100:U100"/>
+    <mergeCell ref="B115:F115"/>
+    <mergeCell ref="G115:K115"/>
+    <mergeCell ref="L115:P115"/>
+    <mergeCell ref="Q115:U115"/>
+    <mergeCell ref="B130:F130"/>
+    <mergeCell ref="G130:K130"/>
+    <mergeCell ref="L130:P130"/>
+    <mergeCell ref="Q130:U130"/>
+    <mergeCell ref="B145:F145"/>
+    <mergeCell ref="G145:K145"/>
+    <mergeCell ref="L145:P145"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -31931,22 +31931,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:53" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="AG1" s="481" t="s">
+      <c r="AG1" s="508" t="s">
         <v>122</v>
       </c>
-      <c r="AH1" s="481" t="s">
+      <c r="AH1" s="508" t="s">
         <v>57</v>
       </c>
-      <c r="AI1" s="481" t="s">
+      <c r="AI1" s="508" t="s">
         <v>52</v>
       </c>
-      <c r="AJ1" s="481" t="s">
+      <c r="AJ1" s="508" t="s">
         <v>122</v>
       </c>
-      <c r="AK1" s="481" t="s">
+      <c r="AK1" s="508" t="s">
         <v>57</v>
       </c>
-      <c r="AL1" s="481" t="s">
+      <c r="AL1" s="508" t="s">
         <v>52</v>
       </c>
     </row>
@@ -32023,23 +32023,23 @@
       <c r="Y2" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="AB2" s="478" t="s">
+      <c r="AB2" s="515" t="s">
         <v>25</v>
       </c>
-      <c r="AC2" s="479"/>
-      <c r="AD2" s="482" t="s">
+      <c r="AC2" s="521"/>
+      <c r="AD2" s="475" t="s">
         <v>58</v>
       </c>
-      <c r="AE2" s="482"/>
+      <c r="AE2" s="475"/>
       <c r="AF2" s="97" t="s">
         <v>97</v>
       </c>
-      <c r="AG2" s="481"/>
-      <c r="AH2" s="481"/>
-      <c r="AI2" s="481"/>
-      <c r="AJ2" s="481"/>
-      <c r="AK2" s="481"/>
-      <c r="AL2" s="481"/>
+      <c r="AG2" s="508"/>
+      <c r="AH2" s="508"/>
+      <c r="AI2" s="508"/>
+      <c r="AJ2" s="508"/>
+      <c r="AK2" s="508"/>
+      <c r="AL2" s="508"/>
     </row>
     <row r="3" spans="2:53" x14ac:dyDescent="0.25">
       <c r="B3" s="14">
@@ -32472,52 +32472,19 @@
       <c r="AA6" s="61" t="s">
         <v>30</v>
       </c>
-      <c r="AB6" s="62">
-        <v>10.304</v>
-      </c>
+      <c r="AB6" s="62"/>
       <c r="AC6" s="382"/>
-      <c r="AD6" s="246">
-        <f>SUM(C72:C74)</f>
-        <v>1.5595000000000001</v>
-      </c>
-      <c r="AE6" s="246">
-        <f>SUM(C75:C78)</f>
-        <v>7.0016999999999996</v>
-      </c>
-      <c r="AF6" s="384">
-        <v>4.8148000000000017</v>
-      </c>
-      <c r="AG6" s="213">
-        <f t="shared" si="0"/>
-        <v>1.4248532844281436</v>
-      </c>
-      <c r="AH6" s="88">
-        <f t="shared" si="1"/>
-        <v>3.2029096365455167</v>
-      </c>
-      <c r="AI6" s="377">
-        <f t="shared" si="2"/>
-        <v>0.18703707902634226</v>
-      </c>
-      <c r="AJ6" s="85">
-        <f>SUM(G34:G46)</f>
-        <v>29.593197732577533</v>
-      </c>
-      <c r="AK6" s="85">
-        <f>SUM(G14:G33)</f>
-        <v>66.522174058019345</v>
-      </c>
-      <c r="AL6" s="85">
-        <v>3.8846282094031355</v>
-      </c>
-      <c r="AM6" s="397">
-        <f t="shared" si="3"/>
-        <v>4.8148000000000026</v>
-      </c>
-      <c r="AN6" s="397">
-        <f t="shared" si="4"/>
-        <v>11.951146715571859</v>
-      </c>
+      <c r="AD6" s="246"/>
+      <c r="AE6" s="246"/>
+      <c r="AF6" s="384"/>
+      <c r="AG6" s="213"/>
+      <c r="AH6" s="88"/>
+      <c r="AI6" s="377"/>
+      <c r="AJ6" s="85"/>
+      <c r="AK6" s="85"/>
+      <c r="AL6" s="85"/>
+      <c r="AM6" s="397"/>
+      <c r="AN6" s="397"/>
     </row>
     <row r="7" spans="2:53" x14ac:dyDescent="0.25">
       <c r="B7" s="28">
@@ -33558,22 +33525,22 @@
       <c r="Y15" s="364">
         <v>1.0235026535253984</v>
       </c>
-      <c r="AG15" s="481" t="s">
+      <c r="AG15" s="508" t="s">
         <v>122</v>
       </c>
-      <c r="AH15" s="481" t="s">
+      <c r="AH15" s="508" t="s">
         <v>57</v>
       </c>
-      <c r="AI15" s="481" t="s">
+      <c r="AI15" s="508" t="s">
         <v>52</v>
       </c>
-      <c r="AJ15" s="481" t="s">
+      <c r="AJ15" s="508" t="s">
         <v>122</v>
       </c>
-      <c r="AK15" s="481" t="s">
+      <c r="AK15" s="508" t="s">
         <v>57</v>
       </c>
-      <c r="AL15" s="481" t="s">
+      <c r="AL15" s="508" t="s">
         <v>52</v>
       </c>
       <c r="AM15" s="397"/>
@@ -33650,23 +33617,23 @@
       <c r="Y16" s="364">
         <v>1.0708870356330553</v>
       </c>
-      <c r="AB16" s="478" t="s">
+      <c r="AB16" s="515" t="s">
         <v>40</v>
       </c>
-      <c r="AC16" s="480"/>
-      <c r="AD16" s="482" t="s">
+      <c r="AC16" s="516"/>
+      <c r="AD16" s="475" t="s">
         <v>58</v>
       </c>
-      <c r="AE16" s="482"/>
+      <c r="AE16" s="475"/>
       <c r="AF16" s="97" t="s">
         <v>97</v>
       </c>
-      <c r="AG16" s="481"/>
-      <c r="AH16" s="481"/>
-      <c r="AI16" s="481"/>
-      <c r="AJ16" s="481"/>
-      <c r="AK16" s="481"/>
-      <c r="AL16" s="481"/>
+      <c r="AG16" s="508"/>
+      <c r="AH16" s="508"/>
+      <c r="AI16" s="508"/>
+      <c r="AJ16" s="508"/>
+      <c r="AK16" s="508"/>
+      <c r="AL16" s="508"/>
       <c r="AM16" s="397"/>
       <c r="AN16" s="397"/>
     </row>
@@ -34215,52 +34182,19 @@
       <c r="AA21" s="63" t="s">
         <v>44</v>
       </c>
-      <c r="AB21" s="64">
-        <v>19.3034</v>
-      </c>
+      <c r="AB21" s="64"/>
       <c r="AC21" s="373"/>
-      <c r="AD21" s="216">
-        <f>SUM(C87:C89)</f>
-        <v>4.3765000000000001</v>
-      </c>
-      <c r="AE21" s="216">
-        <f>SUM(C90:C93)</f>
-        <v>11.661999999999999</v>
-      </c>
-      <c r="AF21" s="221">
-        <v>8.3796999999999997</v>
-      </c>
-      <c r="AG21" s="88">
-        <f>AJ21*AF21/100</f>
-        <v>0.71701174606419926</v>
-      </c>
-      <c r="AH21" s="88">
-        <f>AF21*AK21/100</f>
-        <v>7.1058690962993243</v>
-      </c>
-      <c r="AI21" s="377">
-        <f>AF21*AL21/100</f>
-        <v>0.55681915763647494</v>
-      </c>
-      <c r="AJ21" s="85">
-        <f>SUM(I34:I46)</f>
-        <v>8.5565324064608426</v>
-      </c>
-      <c r="AK21" s="85">
-        <f>SUM(I14:I33)</f>
-        <v>84.798609691269661</v>
-      </c>
-      <c r="AL21" s="85">
-        <v>6.6448579022694725</v>
-      </c>
-      <c r="AM21" s="397">
-        <f t="shared" si="8"/>
-        <v>8.3796999999999979</v>
-      </c>
-      <c r="AN21" s="397">
-        <f>SUM(AD21:AE21,AH21:AI21)</f>
-        <v>23.701188253935797</v>
-      </c>
+      <c r="AD21" s="216"/>
+      <c r="AE21" s="216"/>
+      <c r="AF21" s="221"/>
+      <c r="AG21" s="88"/>
+      <c r="AH21" s="88"/>
+      <c r="AI21" s="377"/>
+      <c r="AJ21" s="85"/>
+      <c r="AK21" s="85"/>
+      <c r="AL21" s="85"/>
+      <c r="AM21" s="397"/>
+      <c r="AN21" s="397"/>
     </row>
     <row r="22" spans="2:40" x14ac:dyDescent="0.25">
       <c r="B22" s="28">
@@ -35325,14 +35259,14 @@
       <c r="Y31" s="364">
         <v>6.6148597422289619</v>
       </c>
-      <c r="AA31" s="476" t="s">
+      <c r="AA31" s="519" t="s">
         <v>25</v>
       </c>
-      <c r="AB31" s="476"/>
-      <c r="AC31" s="477" t="s">
+      <c r="AB31" s="519"/>
+      <c r="AC31" s="520" t="s">
         <v>40</v>
       </c>
-      <c r="AD31" s="477"/>
+      <c r="AD31" s="520"/>
       <c r="AJ31" s="229" t="s">
         <v>73</v>
       </c>
@@ -35651,19 +35585,19 @@
       </c>
       <c r="AK34" s="239">
         <f>AD20-AD6</f>
-        <v>4.7496999999999998</v>
+        <v>6.3091999999999997</v>
       </c>
       <c r="AL34" s="239">
         <f>AE20-AE6</f>
-        <v>-0.38919999999999977</v>
+        <v>6.6124999999999998</v>
       </c>
       <c r="AM34" s="239">
         <f>AH20-AH6</f>
-        <v>0.77072804517574856</v>
+        <v>3.9736376817212653</v>
       </c>
       <c r="AN34" s="239">
         <f>AI20-AI6</f>
-        <v>4.7747439937281033E-2</v>
+        <v>0.23478451896362329</v>
       </c>
     </row>
     <row r="35" spans="2:40" x14ac:dyDescent="0.25">
@@ -35739,11 +35673,11 @@
       </c>
       <c r="AA35" s="60">
         <f t="shared" si="13"/>
-        <v>7.0016999999999996</v>
+        <v>0</v>
       </c>
       <c r="AB35" s="86">
         <f t="shared" si="14"/>
-        <v>1.4248532844281436</v>
+        <v>0</v>
       </c>
       <c r="AC35" s="66">
         <f t="shared" si="15"/>
@@ -35758,19 +35692,19 @@
       </c>
       <c r="AK35" s="239">
         <f>AD7-AD21</f>
-        <v>-3.8315999999999999</v>
+        <v>0.54489999999999994</v>
       </c>
       <c r="AL35" s="239">
         <f>AE7-AE21</f>
-        <v>-8.5400999999999989</v>
+        <v>3.1219000000000001</v>
       </c>
       <c r="AM35" s="239">
         <f t="shared" si="12"/>
-        <v>5.2843239712230581</v>
+        <v>-1.8215451250762664</v>
       </c>
       <c r="AN35" s="239">
         <f>AI21-AI7</f>
-        <v>0.44310253774629799</v>
+        <v>-0.11371661989017695</v>
       </c>
     </row>
     <row r="36" spans="2:40" x14ac:dyDescent="0.25">
@@ -35846,7 +35780,7 @@
       </c>
       <c r="AA36" s="60">
         <f>AE21</f>
-        <v>11.661999999999999</v>
+        <v>0</v>
       </c>
       <c r="AB36" s="86">
         <f t="shared" si="14"/>
@@ -35858,7 +35792,7 @@
       </c>
       <c r="AD36" s="87">
         <f t="shared" si="9"/>
-        <v>0.71701174606419926</v>
+        <v>0</v>
       </c>
       <c r="AJ36" s="233" t="s">
         <v>80</v>
@@ -36842,11 +36776,11 @@
       </c>
       <c r="AK46" s="220">
         <f t="shared" si="18"/>
-        <v>4.8309999999999995</v>
+        <v>15.135</v>
       </c>
       <c r="AL46" s="220">
         <f t="shared" si="19"/>
-        <v>5.1789754851130283</v>
+        <v>17.130122200684887</v>
       </c>
     </row>
     <row r="47" spans="2:40" x14ac:dyDescent="0.25">
@@ -36928,11 +36862,11 @@
       </c>
       <c r="AK47" s="222">
         <f>AB7-AB21</f>
-        <v>-14.6675</v>
+        <v>4.6359000000000004</v>
       </c>
       <c r="AL47" s="222">
         <f t="shared" si="19"/>
-        <v>18.099126508969356</v>
+        <v>-5.6020617449664432</v>
       </c>
     </row>
     <row r="48" spans="2:40" x14ac:dyDescent="0.25">
@@ -36949,10 +36883,10 @@
       </c>
     </row>
     <row r="49" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="AB49" s="482" t="s">
+      <c r="AB49" s="475" t="s">
         <v>137</v>
       </c>
-      <c r="AC49" s="482"/>
+      <c r="AC49" s="475"/>
       <c r="AJ49" s="233" t="s">
         <v>81</v>
       </c>
@@ -37015,7 +36949,7 @@
         <v>1.1408</v>
       </c>
       <c r="AF51" s="85">
-        <f t="shared" ref="AF51" si="20">AVERAGE(AE4:AE5)</f>
+        <f>AVERAGE(AE4:AE5)</f>
         <v>6.6535499999999992</v>
       </c>
       <c r="AG51" s="85">
@@ -37043,29 +36977,29 @@
       <c r="AA52" s="61" t="s">
         <v>107</v>
       </c>
-      <c r="AB52" s="85">
+      <c r="AB52" s="85" t="e">
         <f>AVERAGE(AB6)</f>
-        <v>10.304</v>
-      </c>
-      <c r="AC52" s="85">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC52" s="85" t="e">
         <f>AVERAGE(AN6)</f>
-        <v>11.951146715571859</v>
-      </c>
-      <c r="AE52" s="85">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE52" s="85" t="e">
         <f>AVERAGE(AD6)</f>
-        <v>1.5595000000000001</v>
-      </c>
-      <c r="AF52" s="85">
-        <f t="shared" ref="AF52" si="21">AVERAGE(AE6)</f>
-        <v>7.0016999999999996</v>
-      </c>
-      <c r="AG52" s="85">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF52" s="85" t="e">
+        <f t="shared" ref="AF52" si="20">AVERAGE(AE6)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG52" s="85" t="e">
         <f>AVERAGE(AH6)</f>
-        <v>3.2029096365455167</v>
-      </c>
-      <c r="AH52" s="85">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH52" s="85" t="e">
         <f>AVERAGE(AI6)</f>
-        <v>0.18703707902634226</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="AJ52" s="235" t="s">
         <v>85</v>
@@ -37098,11 +37032,11 @@
       </c>
       <c r="AE53" s="85">
         <f>AD21</f>
-        <v>4.3765000000000001</v>
+        <v>0</v>
       </c>
       <c r="AF53" s="85">
         <f>AE21</f>
-        <v>11.661999999999999</v>
+        <v>0</v>
       </c>
       <c r="AG53" s="85">
         <f>AH7</f>
@@ -37142,7 +37076,7 @@
         <v>6.3520000000000003</v>
       </c>
       <c r="AF54" s="85">
-        <f t="shared" ref="AF54" si="22">AVERAGE(AE8:AE9)</f>
+        <f t="shared" ref="AF54" si="21">AVERAGE(AE8:AE9)</f>
         <v>9.2189999999999994</v>
       </c>
       <c r="AG54" s="85">
@@ -37156,34 +37090,34 @@
       <c r="AN54" s="85"/>
     </row>
     <row r="55" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B55" s="518" t="s">
+      <c r="B55" s="523" t="s">
         <v>1</v>
       </c>
-      <c r="C55" s="519"/>
-      <c r="D55" s="519"/>
-      <c r="E55" s="519"/>
-      <c r="F55" s="520"/>
-      <c r="G55" s="518" t="s">
+      <c r="C55" s="524"/>
+      <c r="D55" s="524"/>
+      <c r="E55" s="524"/>
+      <c r="F55" s="525"/>
+      <c r="G55" s="523" t="s">
         <v>2</v>
       </c>
-      <c r="H55" s="519"/>
-      <c r="I55" s="519"/>
-      <c r="J55" s="519"/>
-      <c r="K55" s="520"/>
-      <c r="L55" s="518" t="s">
+      <c r="H55" s="524"/>
+      <c r="I55" s="524"/>
+      <c r="J55" s="524"/>
+      <c r="K55" s="525"/>
+      <c r="L55" s="523" t="s">
         <v>3</v>
       </c>
-      <c r="M55" s="519"/>
-      <c r="N55" s="519"/>
-      <c r="O55" s="519"/>
-      <c r="P55" s="520"/>
-      <c r="Q55" s="518" t="s">
+      <c r="M55" s="524"/>
+      <c r="N55" s="524"/>
+      <c r="O55" s="524"/>
+      <c r="P55" s="525"/>
+      <c r="Q55" s="523" t="s">
         <v>4</v>
       </c>
-      <c r="R55" s="519"/>
-      <c r="S55" s="519"/>
-      <c r="T55" s="519"/>
-      <c r="U55" s="520"/>
+      <c r="R55" s="524"/>
+      <c r="S55" s="524"/>
+      <c r="T55" s="524"/>
+      <c r="U55" s="525"/>
       <c r="AA55" s="67" t="s">
         <v>110</v>
       </c>
@@ -37200,7 +37134,7 @@
         <v>6.3075000000000001</v>
       </c>
       <c r="AF55" s="85">
-        <f t="shared" ref="AF55" si="23">AVERAGE(AE10)</f>
+        <f t="shared" ref="AF55" si="22">AVERAGE(AE10)</f>
         <v>6.8244000000000007</v>
       </c>
       <c r="AG55" s="85">
@@ -37290,7 +37224,7 @@
         <v>2.2075499999999999</v>
       </c>
       <c r="AF56" s="85">
-        <f t="shared" ref="AF56" si="24">AVERAGE(AE11:AE12)</f>
+        <f t="shared" ref="AF56" si="23">AVERAGE(AE11:AE12)</f>
         <v>7.8794499999999994</v>
       </c>
       <c r="AG56" s="85">
@@ -37380,7 +37314,7 @@
         <v>1.2798999999999998</v>
       </c>
       <c r="AF57" s="85">
-        <f t="shared" ref="AF57" si="25">AVERAGE(AE13:AE14)</f>
+        <f t="shared" ref="AF57" si="24">AVERAGE(AE13:AE14)</f>
         <v>9.4603999999999999</v>
       </c>
       <c r="AG57" s="85">
@@ -37453,17 +37387,17 @@
       <c r="U58" s="250">
         <v>93.215838326871108</v>
       </c>
-      <c r="AB58" s="478" t="s">
+      <c r="AB58" s="515" t="s">
         <v>138</v>
       </c>
-      <c r="AC58" s="480"/>
-      <c r="AI58" s="493" t="s">
+      <c r="AC58" s="516"/>
+      <c r="AI58" s="517" t="s">
         <v>136</v>
       </c>
-      <c r="AJ58" s="493"/>
-      <c r="AK58" s="493"/>
-      <c r="AL58" s="493"/>
-      <c r="AM58" s="493"/>
+      <c r="AJ58" s="517"/>
+      <c r="AK58" s="517"/>
+      <c r="AL58" s="517"/>
+      <c r="AM58" s="517"/>
     </row>
     <row r="59" spans="2:41" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B59" s="170">
@@ -37657,11 +37591,11 @@
         <v>0.27329999999999988</v>
       </c>
       <c r="AK60" s="239">
-        <f t="shared" ref="AK60:AM66" si="26">AF60-AF51</f>
+        <f>AF60-AF51</f>
         <v>3.428090000000001</v>
       </c>
       <c r="AL60" s="239">
-        <f t="shared" si="26"/>
+        <f t="shared" ref="AK60:AM66" si="25">AG60-AG51</f>
         <v>1.3766493955717056</v>
       </c>
       <c r="AM60" s="239">
@@ -37747,7 +37681,7 @@
         <v>6.3091999999999997</v>
       </c>
       <c r="AF61" s="85">
-        <f t="shared" ref="AF61" si="27">AVERAGE(AE20)</f>
+        <f t="shared" ref="AF61" si="26">AVERAGE(AE20)</f>
         <v>6.6124999999999998</v>
       </c>
       <c r="AG61" s="85">
@@ -37761,21 +37695,21 @@
       <c r="AI61" s="61" t="s">
         <v>107</v>
       </c>
-      <c r="AJ61" s="239">
-        <f t="shared" ref="AJ61:AJ65" si="28">AE61-AE52</f>
-        <v>4.7496999999999998</v>
-      </c>
-      <c r="AK61" s="239">
-        <f t="shared" si="26"/>
-        <v>-0.38919999999999977</v>
-      </c>
-      <c r="AL61" s="239">
-        <f t="shared" si="26"/>
-        <v>0.77072804517574856</v>
-      </c>
-      <c r="AM61" s="239">
-        <f t="shared" si="26"/>
-        <v>4.7747439937281033E-2</v>
+      <c r="AJ61" s="239" t="e">
+        <f t="shared" ref="AJ61:AJ65" si="27">AE61-AE52</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AK61" s="239" t="e">
+        <f t="shared" si="25"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AL61" s="239" t="e">
+        <f t="shared" si="25"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AM61" s="239" t="e">
+        <f t="shared" si="25"/>
+        <v>#DIV/0!</v>
       </c>
       <c r="AO61" s="85"/>
     </row>
@@ -37849,13 +37783,13 @@
       <c r="AA62" s="63" t="s">
         <v>108</v>
       </c>
-      <c r="AB62" s="85">
+      <c r="AB62" s="85" t="e">
         <f>AVERAGE(AB21)</f>
-        <v>19.3034</v>
-      </c>
-      <c r="AC62" s="85">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC62" s="85" t="e">
         <f>AVERAGE(AN21)</f>
-        <v>23.701188253935797</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="AE62" s="85">
         <f>AVERAGE(AD7)</f>
@@ -37865,32 +37799,32 @@
         <f>AVERAGE(AE7)</f>
         <v>3.1219000000000001</v>
       </c>
-      <c r="AG62" s="85">
+      <c r="AG62" s="85" t="e">
         <f>AVERAGE(AH21)</f>
-        <v>7.1058690962993243</v>
-      </c>
-      <c r="AH62" s="85">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH62" s="85" t="e">
         <f>AVERAGE(AI21)</f>
-        <v>0.55681915763647494</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="AI62" s="63" t="s">
         <v>108</v>
       </c>
       <c r="AJ62" s="239">
         <f>AE62-AE53</f>
-        <v>-3.8315999999999999</v>
+        <v>0.54489999999999994</v>
       </c>
       <c r="AK62" s="239">
-        <f t="shared" si="26"/>
-        <v>-8.5400999999999989</v>
-      </c>
-      <c r="AL62" s="239">
-        <f t="shared" si="26"/>
-        <v>5.2843239712230581</v>
-      </c>
-      <c r="AM62" s="239">
-        <f t="shared" si="26"/>
-        <v>0.44310253774629799</v>
+        <f t="shared" si="25"/>
+        <v>3.1219000000000001</v>
+      </c>
+      <c r="AL62" s="239" t="e">
+        <f t="shared" si="25"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AM62" s="239" t="e">
+        <f t="shared" si="25"/>
+        <v>#DIV/0!</v>
       </c>
       <c r="AO62" s="85"/>
     </row>
@@ -37978,7 +37912,7 @@
         <v>3.1256500000000003</v>
       </c>
       <c r="AF63" s="85">
-        <f t="shared" ref="AF63" si="29">AVERAGE(AE22:AE23)</f>
+        <f t="shared" ref="AF63" si="28">AVERAGE(AE22:AE23)</f>
         <v>7.1271000000000004</v>
       </c>
       <c r="AG63" s="85">
@@ -37993,19 +37927,19 @@
         <v>109</v>
       </c>
       <c r="AJ63" s="239">
-        <f t="shared" si="28"/>
+        <f t="shared" si="27"/>
         <v>-3.2263500000000001</v>
       </c>
       <c r="AK63" s="239">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>-2.091899999999999</v>
       </c>
       <c r="AL63" s="239">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>-0.3989000650117589</v>
       </c>
       <c r="AM63" s="239">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>-8.1408390169192879E-2</v>
       </c>
       <c r="AO63" s="85"/>
@@ -38094,7 +38028,7 @@
         <v>2.1496</v>
       </c>
       <c r="AF64" s="85">
-        <f t="shared" ref="AF64" si="30">AVERAGE(AE24:AE25)</f>
+        <f t="shared" ref="AF64" si="29">AVERAGE(AE24:AE25)</f>
         <v>8.3337000000000003</v>
       </c>
       <c r="AG64" s="85">
@@ -38109,19 +38043,19 @@
         <v>110</v>
       </c>
       <c r="AJ64" s="239">
-        <f t="shared" si="28"/>
+        <f t="shared" si="27"/>
         <v>-4.1578999999999997</v>
       </c>
       <c r="AK64" s="239">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>1.5092999999999996</v>
       </c>
       <c r="AL64" s="239">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>1.4359332002046834</v>
       </c>
       <c r="AM64" s="239">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>0.10111553238929508</v>
       </c>
       <c r="AO64" s="85"/>
@@ -38210,7 +38144,7 @@
         <v>0.79820000000000002</v>
       </c>
       <c r="AF65" s="85">
-        <f t="shared" ref="AF65" si="31">AVERAGE(AE26:AE27)</f>
+        <f t="shared" ref="AF65" si="30">AVERAGE(AE26:AE27)</f>
         <v>7.6038999999999994</v>
       </c>
       <c r="AG65" s="85">
@@ -38225,19 +38159,19 @@
         <v>111</v>
       </c>
       <c r="AJ65" s="239">
-        <f t="shared" si="28"/>
+        <f t="shared" si="27"/>
         <v>-1.4093499999999999</v>
       </c>
       <c r="AK65" s="239">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>-0.27554999999999996</v>
       </c>
       <c r="AL65" s="239">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>0.57420834985419233</v>
       </c>
       <c r="AM65" s="239">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>6.4538108255397297E-2</v>
       </c>
       <c r="AO65" s="85"/>
@@ -38326,7 +38260,7 @@
         <v>1.4544000000000001</v>
       </c>
       <c r="AF66" s="85">
-        <f t="shared" ref="AF66" si="32">AVERAGE(AE28)</f>
+        <f t="shared" ref="AF66" si="31">AVERAGE(AE28)</f>
         <v>9.8343000000000007</v>
       </c>
       <c r="AG66" s="85">
@@ -38345,15 +38279,15 @@
         <v>0.17450000000000032</v>
       </c>
       <c r="AK66" s="239">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>0.37390000000000079</v>
       </c>
       <c r="AL66" s="239">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>1.356578484203486</v>
       </c>
       <c r="AM66" s="239">
-        <f t="shared" si="26"/>
+        <f t="shared" si="25"/>
         <v>-9.0322894183338387E-2</v>
       </c>
       <c r="AO66" s="85"/>
@@ -38483,20 +38417,20 @@
       </c>
     </row>
     <row r="70" spans="2:41" x14ac:dyDescent="0.25">
-      <c r="B70" s="506" t="s">
+      <c r="B70" s="487" t="s">
         <v>5</v>
       </c>
-      <c r="C70" s="507"/>
-      <c r="D70" s="507"/>
-      <c r="E70" s="507"/>
-      <c r="F70" s="508"/>
-      <c r="G70" s="506" t="s">
+      <c r="C70" s="488"/>
+      <c r="D70" s="488"/>
+      <c r="E70" s="488"/>
+      <c r="F70" s="489"/>
+      <c r="G70" s="487" t="s">
         <v>6</v>
       </c>
-      <c r="H70" s="507"/>
-      <c r="I70" s="507"/>
-      <c r="J70" s="507"/>
-      <c r="K70" s="508"/>
+      <c r="H70" s="488"/>
+      <c r="I70" s="488"/>
+      <c r="J70" s="488"/>
+      <c r="K70" s="489"/>
       <c r="R70" s="83"/>
       <c r="S70" s="83"/>
       <c r="V70" s="83"/>
@@ -38506,13 +38440,13 @@
       <c r="AJ70" s="61" t="s">
         <v>107</v>
       </c>
-      <c r="AK70" s="85">
-        <f t="shared" ref="AK70:AL75" si="33">AB61-AB52</f>
-        <v>4.8309999999999995</v>
-      </c>
-      <c r="AL70" s="85">
+      <c r="AK70" s="85" t="e">
+        <f t="shared" ref="AK70:AL75" si="32">AB61-AB52</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AL70" s="85" t="e">
         <f>AC61-AC52</f>
-        <v>5.1789754851130283</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="71" spans="2:41" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -38557,13 +38491,13 @@
       <c r="AJ71" s="63" t="s">
         <v>108</v>
       </c>
-      <c r="AK71" s="85">
-        <f t="shared" si="33"/>
-        <v>14.6675</v>
-      </c>
-      <c r="AL71" s="85">
+      <c r="AK71" s="85" t="e">
+        <f t="shared" si="32"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AL71" s="85" t="e">
         <f>AC62-AC53</f>
-        <v>18.099126508969356</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="72" spans="2:41" x14ac:dyDescent="0.25">
@@ -38617,7 +38551,7 @@
         <v>109</v>
       </c>
       <c r="AK72" s="85">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>-5.3126999999999995</v>
       </c>
       <c r="AL72" s="85">
@@ -38677,11 +38611,11 @@
         <v>110</v>
       </c>
       <c r="AK73" s="85">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>-1.8184000000000022</v>
       </c>
       <c r="AL73" s="85">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>-1.1115512674060248</v>
       </c>
     </row>
@@ -38733,11 +38667,11 @@
         <v>111</v>
       </c>
       <c r="AK74" s="85">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>-1.2214999999999989</v>
       </c>
       <c r="AL74" s="85">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>-1.0461535418904102</v>
       </c>
     </row>
@@ -38786,11 +38720,11 @@
         <v>112</v>
       </c>
       <c r="AK75" s="85">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>0.77880000000000038</v>
       </c>
       <c r="AL75" s="85">
-        <f t="shared" si="33"/>
+        <f t="shared" si="32"/>
         <v>1.8146555900201484</v>
       </c>
     </row>
@@ -39112,20 +39046,20 @@
     </row>
     <row r="84" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="85" spans="2:29" x14ac:dyDescent="0.25">
-      <c r="B85" s="515" t="s">
+      <c r="B85" s="526" t="s">
         <v>7</v>
       </c>
-      <c r="C85" s="516"/>
-      <c r="D85" s="516"/>
-      <c r="E85" s="516"/>
-      <c r="F85" s="517"/>
-      <c r="G85" s="515" t="s">
+      <c r="C85" s="527"/>
+      <c r="D85" s="527"/>
+      <c r="E85" s="527"/>
+      <c r="F85" s="528"/>
+      <c r="G85" s="526" t="s">
         <v>8</v>
       </c>
-      <c r="H85" s="516"/>
-      <c r="I85" s="516"/>
-      <c r="J85" s="516"/>
-      <c r="K85" s="517"/>
+      <c r="H85" s="527"/>
+      <c r="I85" s="527"/>
+      <c r="J85" s="527"/>
+      <c r="K85" s="528"/>
       <c r="M85" t="s">
         <v>119</v>
       </c>
@@ -39555,34 +39489,34 @@
     </row>
     <row r="99" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="100" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B100" s="497" t="s">
+      <c r="B100" s="499" t="s">
         <v>9</v>
       </c>
-      <c r="C100" s="498"/>
-      <c r="D100" s="498"/>
-      <c r="E100" s="498"/>
-      <c r="F100" s="499"/>
-      <c r="G100" s="497" t="s">
+      <c r="C100" s="500"/>
+      <c r="D100" s="500"/>
+      <c r="E100" s="500"/>
+      <c r="F100" s="501"/>
+      <c r="G100" s="499" t="s">
         <v>10</v>
       </c>
-      <c r="H100" s="498"/>
-      <c r="I100" s="498"/>
-      <c r="J100" s="498"/>
-      <c r="K100" s="499"/>
-      <c r="L100" s="497" t="s">
+      <c r="H100" s="500"/>
+      <c r="I100" s="500"/>
+      <c r="J100" s="500"/>
+      <c r="K100" s="501"/>
+      <c r="L100" s="499" t="s">
         <v>11</v>
       </c>
-      <c r="M100" s="498"/>
-      <c r="N100" s="498"/>
-      <c r="O100" s="498"/>
-      <c r="P100" s="499"/>
-      <c r="Q100" s="497" t="s">
+      <c r="M100" s="500"/>
+      <c r="N100" s="500"/>
+      <c r="O100" s="500"/>
+      <c r="P100" s="501"/>
+      <c r="Q100" s="499" t="s">
         <v>12</v>
       </c>
-      <c r="R100" s="498"/>
-      <c r="S100" s="498"/>
-      <c r="T100" s="498"/>
-      <c r="U100" s="499"/>
+      <c r="R100" s="500"/>
+      <c r="S100" s="500"/>
+      <c r="T100" s="500"/>
+      <c r="U100" s="501"/>
     </row>
     <row r="101" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B101" s="183" t="s">
@@ -40404,34 +40338,34 @@
     </row>
     <row r="114" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="115" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B115" s="500" t="s">
+      <c r="B115" s="502" t="s">
         <v>13</v>
       </c>
-      <c r="C115" s="501"/>
-      <c r="D115" s="501"/>
-      <c r="E115" s="501"/>
-      <c r="F115" s="502"/>
-      <c r="G115" s="503" t="s">
+      <c r="C115" s="503"/>
+      <c r="D115" s="503"/>
+      <c r="E115" s="503"/>
+      <c r="F115" s="504"/>
+      <c r="G115" s="505" t="s">
         <v>14</v>
       </c>
-      <c r="H115" s="504"/>
-      <c r="I115" s="504"/>
-      <c r="J115" s="504"/>
-      <c r="K115" s="505"/>
-      <c r="L115" s="503" t="s">
+      <c r="H115" s="506"/>
+      <c r="I115" s="506"/>
+      <c r="J115" s="506"/>
+      <c r="K115" s="507"/>
+      <c r="L115" s="505" t="s">
         <v>15</v>
       </c>
-      <c r="M115" s="504"/>
-      <c r="N115" s="504"/>
-      <c r="O115" s="504"/>
-      <c r="P115" s="505"/>
-      <c r="Q115" s="503" t="s">
+      <c r="M115" s="506"/>
+      <c r="N115" s="506"/>
+      <c r="O115" s="506"/>
+      <c r="P115" s="507"/>
+      <c r="Q115" s="505" t="s">
         <v>16</v>
       </c>
-      <c r="R115" s="504"/>
-      <c r="S115" s="504"/>
-      <c r="T115" s="504"/>
-      <c r="U115" s="505"/>
+      <c r="R115" s="506"/>
+      <c r="S115" s="506"/>
+      <c r="T115" s="506"/>
+      <c r="U115" s="507"/>
     </row>
     <row r="116" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B116" s="193" t="s">
@@ -41130,34 +41064,34 @@
     </row>
     <row r="129" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="130" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B130" s="506" t="s">
+      <c r="B130" s="487" t="s">
         <v>17</v>
       </c>
-      <c r="C130" s="507"/>
-      <c r="D130" s="507"/>
-      <c r="E130" s="507"/>
-      <c r="F130" s="508"/>
-      <c r="G130" s="506" t="s">
+      <c r="C130" s="488"/>
+      <c r="D130" s="488"/>
+      <c r="E130" s="488"/>
+      <c r="F130" s="489"/>
+      <c r="G130" s="487" t="s">
         <v>18</v>
       </c>
-      <c r="H130" s="507"/>
-      <c r="I130" s="507"/>
-      <c r="J130" s="507"/>
-      <c r="K130" s="508"/>
-      <c r="L130" s="506" t="s">
+      <c r="H130" s="488"/>
+      <c r="I130" s="488"/>
+      <c r="J130" s="488"/>
+      <c r="K130" s="489"/>
+      <c r="L130" s="487" t="s">
         <v>19</v>
       </c>
-      <c r="M130" s="507"/>
-      <c r="N130" s="507"/>
-      <c r="O130" s="507"/>
-      <c r="P130" s="508"/>
-      <c r="Q130" s="506" t="s">
+      <c r="M130" s="488"/>
+      <c r="N130" s="488"/>
+      <c r="O130" s="488"/>
+      <c r="P130" s="489"/>
+      <c r="Q130" s="487" t="s">
         <v>20</v>
       </c>
-      <c r="R130" s="507"/>
-      <c r="S130" s="507"/>
-      <c r="T130" s="507"/>
-      <c r="U130" s="508"/>
+      <c r="R130" s="488"/>
+      <c r="S130" s="488"/>
+      <c r="T130" s="488"/>
+      <c r="U130" s="489"/>
     </row>
     <row r="131" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B131" s="150" t="s">
@@ -41979,27 +41913,27 @@
     </row>
     <row r="144" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="145" spans="2:24" x14ac:dyDescent="0.25">
-      <c r="B145" s="512" t="s">
+      <c r="B145" s="493" t="s">
         <v>21</v>
       </c>
-      <c r="C145" s="513"/>
-      <c r="D145" s="513"/>
-      <c r="E145" s="513"/>
-      <c r="F145" s="514"/>
-      <c r="G145" s="512" t="s">
+      <c r="C145" s="494"/>
+      <c r="D145" s="494"/>
+      <c r="E145" s="494"/>
+      <c r="F145" s="495"/>
+      <c r="G145" s="493" t="s">
         <v>22</v>
       </c>
-      <c r="H145" s="513"/>
-      <c r="I145" s="513"/>
-      <c r="J145" s="513"/>
-      <c r="K145" s="514"/>
-      <c r="L145" s="512" t="s">
+      <c r="H145" s="494"/>
+      <c r="I145" s="494"/>
+      <c r="J145" s="494"/>
+      <c r="K145" s="495"/>
+      <c r="L145" s="493" t="s">
         <v>23</v>
       </c>
-      <c r="M145" s="513"/>
-      <c r="N145" s="513"/>
-      <c r="O145" s="513"/>
-      <c r="P145" s="514"/>
+      <c r="M145" s="494"/>
+      <c r="N145" s="494"/>
+      <c r="O145" s="494"/>
+      <c r="P145" s="495"/>
     </row>
     <row r="146" spans="2:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B146" s="203" t="s">
@@ -42625,6 +42559,34 @@
     </row>
   </sheetData>
   <mergeCells count="44">
+    <mergeCell ref="AL1:AL2"/>
+    <mergeCell ref="AB2:AC2"/>
+    <mergeCell ref="AD2:AE2"/>
+    <mergeCell ref="AG1:AG2"/>
+    <mergeCell ref="AH1:AH2"/>
+    <mergeCell ref="AI1:AI2"/>
+    <mergeCell ref="AJ1:AJ2"/>
+    <mergeCell ref="AK1:AK2"/>
+    <mergeCell ref="AK15:AK16"/>
+    <mergeCell ref="AL15:AL16"/>
+    <mergeCell ref="AB16:AC16"/>
+    <mergeCell ref="AD16:AE16"/>
+    <mergeCell ref="AA31:AB31"/>
+    <mergeCell ref="AC31:AD31"/>
+    <mergeCell ref="AJ15:AJ16"/>
+    <mergeCell ref="AG15:AG16"/>
+    <mergeCell ref="AH15:AH16"/>
+    <mergeCell ref="AI15:AI16"/>
+    <mergeCell ref="G85:K85"/>
+    <mergeCell ref="B85:F85"/>
+    <mergeCell ref="B100:F100"/>
+    <mergeCell ref="G100:K100"/>
+    <mergeCell ref="L100:P100"/>
+    <mergeCell ref="G55:K55"/>
+    <mergeCell ref="L55:P55"/>
+    <mergeCell ref="Q55:U55"/>
+    <mergeCell ref="B70:F70"/>
+    <mergeCell ref="G70:K70"/>
     <mergeCell ref="AB49:AC49"/>
     <mergeCell ref="AB58:AC58"/>
     <mergeCell ref="AI58:AM58"/>
@@ -42641,34 +42603,6 @@
     <mergeCell ref="Q130:U130"/>
     <mergeCell ref="Q100:U100"/>
     <mergeCell ref="B55:F55"/>
-    <mergeCell ref="G55:K55"/>
-    <mergeCell ref="L55:P55"/>
-    <mergeCell ref="Q55:U55"/>
-    <mergeCell ref="B70:F70"/>
-    <mergeCell ref="G70:K70"/>
-    <mergeCell ref="G85:K85"/>
-    <mergeCell ref="B85:F85"/>
-    <mergeCell ref="B100:F100"/>
-    <mergeCell ref="G100:K100"/>
-    <mergeCell ref="L100:P100"/>
-    <mergeCell ref="AK15:AK16"/>
-    <mergeCell ref="AL15:AL16"/>
-    <mergeCell ref="AB16:AC16"/>
-    <mergeCell ref="AD16:AE16"/>
-    <mergeCell ref="AA31:AB31"/>
-    <mergeCell ref="AC31:AD31"/>
-    <mergeCell ref="AJ15:AJ16"/>
-    <mergeCell ref="AG15:AG16"/>
-    <mergeCell ref="AH15:AH16"/>
-    <mergeCell ref="AI15:AI16"/>
-    <mergeCell ref="AL1:AL2"/>
-    <mergeCell ref="AB2:AC2"/>
-    <mergeCell ref="AD2:AE2"/>
-    <mergeCell ref="AG1:AG2"/>
-    <mergeCell ref="AH1:AH2"/>
-    <mergeCell ref="AI1:AI2"/>
-    <mergeCell ref="AJ1:AJ2"/>
-    <mergeCell ref="AK1:AK2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -42706,62 +42640,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:60" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="521" t="s">
+      <c r="A1" s="480" t="s">
         <v>92</v>
       </c>
-      <c r="B1" s="524"/>
-      <c r="C1" s="524"/>
-      <c r="D1" s="524"/>
-      <c r="E1" s="524"/>
-      <c r="F1" s="524"/>
-      <c r="G1" s="524"/>
-      <c r="H1" s="524"/>
-      <c r="I1" s="524"/>
-      <c r="J1" s="524"/>
-      <c r="K1" s="524"/>
-      <c r="L1" s="524"/>
-      <c r="M1" s="524"/>
-      <c r="N1" s="523"/>
+      <c r="B1" s="483"/>
+      <c r="C1" s="483"/>
+      <c r="D1" s="483"/>
+      <c r="E1" s="483"/>
+      <c r="F1" s="483"/>
+      <c r="G1" s="483"/>
+      <c r="H1" s="483"/>
+      <c r="I1" s="483"/>
+      <c r="J1" s="483"/>
+      <c r="K1" s="483"/>
+      <c r="L1" s="483"/>
+      <c r="M1" s="483"/>
+      <c r="N1" s="482"/>
     </row>
     <row r="2" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A2" s="439"/>
-      <c r="B2" s="521" t="s">
+      <c r="B2" s="480" t="s">
         <v>104</v>
       </c>
-      <c r="C2" s="522"/>
-      <c r="D2" s="523"/>
-      <c r="E2" s="521" t="s">
+      <c r="C2" s="481"/>
+      <c r="D2" s="482"/>
+      <c r="E2" s="480" t="s">
         <v>101</v>
       </c>
-      <c r="F2" s="522"/>
-      <c r="G2" s="523"/>
-      <c r="H2" s="521" t="s">
+      <c r="F2" s="481"/>
+      <c r="G2" s="482"/>
+      <c r="H2" s="480" t="s">
         <v>103</v>
       </c>
-      <c r="I2" s="522"/>
-      <c r="J2" s="523"/>
-      <c r="K2" s="521" t="s">
+      <c r="I2" s="481"/>
+      <c r="J2" s="482"/>
+      <c r="K2" s="480" t="s">
         <v>72</v>
       </c>
-      <c r="L2" s="522"/>
-      <c r="M2" s="523"/>
+      <c r="L2" s="481"/>
+      <c r="M2" s="482"/>
       <c r="N2" s="440"/>
-      <c r="Q2" s="482" t="s">
+      <c r="Q2" s="475" t="s">
         <v>141</v>
       </c>
-      <c r="R2" s="526"/>
-      <c r="S2" s="526"/>
-      <c r="T2" s="526"/>
-      <c r="U2" s="526"/>
-      <c r="V2" s="526"/>
-      <c r="W2" s="526"/>
-      <c r="X2" s="526"/>
-      <c r="Y2" s="526"/>
-      <c r="Z2" s="526"/>
-      <c r="AA2" s="526"/>
-      <c r="AB2" s="526"/>
-      <c r="AC2" s="526"/>
-      <c r="AD2" s="482"/>
+      <c r="R2" s="476"/>
+      <c r="S2" s="476"/>
+      <c r="T2" s="476"/>
+      <c r="U2" s="476"/>
+      <c r="V2" s="476"/>
+      <c r="W2" s="476"/>
+      <c r="X2" s="476"/>
+      <c r="Y2" s="476"/>
+      <c r="Z2" s="476"/>
+      <c r="AA2" s="476"/>
+      <c r="AB2" s="476"/>
+      <c r="AC2" s="476"/>
+      <c r="AD2" s="475"/>
     </row>
     <row r="3" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A3" s="441" t="s">
@@ -42807,26 +42741,26 @@
         <v>27</v>
       </c>
       <c r="Q3" s="228"/>
-      <c r="R3" s="482" t="s">
+      <c r="R3" s="475" t="s">
         <v>104</v>
       </c>
-      <c r="S3" s="482"/>
-      <c r="T3" s="482"/>
-      <c r="U3" s="482" t="s">
+      <c r="S3" s="475"/>
+      <c r="T3" s="475"/>
+      <c r="U3" s="475" t="s">
         <v>102</v>
       </c>
-      <c r="V3" s="482"/>
-      <c r="W3" s="482"/>
-      <c r="X3" s="482" t="s">
+      <c r="V3" s="475"/>
+      <c r="W3" s="475"/>
+      <c r="X3" s="475" t="s">
         <v>103</v>
       </c>
-      <c r="Y3" s="482"/>
-      <c r="Z3" s="482"/>
-      <c r="AA3" s="482" t="s">
+      <c r="Y3" s="475"/>
+      <c r="Z3" s="475"/>
+      <c r="AA3" s="475" t="s">
         <v>72</v>
       </c>
-      <c r="AB3" s="482"/>
-      <c r="AC3" s="482"/>
+      <c r="AB3" s="475"/>
+      <c r="AC3" s="475"/>
       <c r="AD3" s="244"/>
     </row>
     <row r="4" spans="1:60" x14ac:dyDescent="0.25">
@@ -43814,22 +43748,22 @@
       <c r="N13" s="462">
         <v>-0.16746416727938898</v>
       </c>
-      <c r="Q13" s="482" t="s">
+      <c r="Q13" s="475" t="s">
         <v>142</v>
       </c>
-      <c r="R13" s="526"/>
-      <c r="S13" s="526"/>
-      <c r="T13" s="526"/>
-      <c r="U13" s="526"/>
-      <c r="V13" s="526"/>
-      <c r="W13" s="526"/>
-      <c r="X13" s="526"/>
-      <c r="Y13" s="526"/>
-      <c r="Z13" s="526"/>
-      <c r="AA13" s="526"/>
-      <c r="AB13" s="526"/>
-      <c r="AC13" s="526"/>
-      <c r="AD13" s="482"/>
+      <c r="R13" s="476"/>
+      <c r="S13" s="476"/>
+      <c r="T13" s="476"/>
+      <c r="U13" s="476"/>
+      <c r="V13" s="476"/>
+      <c r="W13" s="476"/>
+      <c r="X13" s="476"/>
+      <c r="Y13" s="476"/>
+      <c r="Z13" s="476"/>
+      <c r="AA13" s="476"/>
+      <c r="AB13" s="476"/>
+      <c r="AC13" s="476"/>
+      <c r="AD13" s="475"/>
     </row>
     <row r="14" spans="1:60" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="449" t="s">
@@ -43887,26 +43821,26 @@
         <v>-3.3378369109007613E-2</v>
       </c>
       <c r="Q14" s="228"/>
-      <c r="R14" s="482" t="s">
+      <c r="R14" s="475" t="s">
         <v>104</v>
       </c>
-      <c r="S14" s="482"/>
-      <c r="T14" s="482"/>
-      <c r="U14" s="482" t="s">
+      <c r="S14" s="475"/>
+      <c r="T14" s="475"/>
+      <c r="U14" s="475" t="s">
         <v>102</v>
       </c>
-      <c r="V14" s="482"/>
-      <c r="W14" s="482"/>
-      <c r="X14" s="482" t="s">
+      <c r="V14" s="475"/>
+      <c r="W14" s="475"/>
+      <c r="X14" s="475" t="s">
         <v>103</v>
       </c>
-      <c r="Y14" s="482"/>
-      <c r="Z14" s="482"/>
-      <c r="AA14" s="482" t="s">
+      <c r="Y14" s="475"/>
+      <c r="Z14" s="475"/>
+      <c r="AA14" s="475" t="s">
         <v>72</v>
       </c>
-      <c r="AB14" s="482"/>
-      <c r="AC14" s="482"/>
+      <c r="AB14" s="475"/>
+      <c r="AC14" s="475"/>
       <c r="AD14" s="244"/>
     </row>
     <row r="15" spans="1:60" x14ac:dyDescent="0.25">
@@ -43959,22 +43893,22 @@
       </c>
     </row>
     <row r="16" spans="1:60" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="525" t="s">
+      <c r="A16" s="478" t="s">
         <v>99</v>
       </c>
-      <c r="B16" s="526"/>
-      <c r="C16" s="526"/>
-      <c r="D16" s="526"/>
-      <c r="E16" s="526"/>
-      <c r="F16" s="526"/>
-      <c r="G16" s="526"/>
-      <c r="H16" s="526"/>
-      <c r="I16" s="526"/>
-      <c r="J16" s="526"/>
-      <c r="K16" s="526"/>
-      <c r="L16" s="526"/>
-      <c r="M16" s="526"/>
-      <c r="N16" s="527"/>
+      <c r="B16" s="476"/>
+      <c r="C16" s="476"/>
+      <c r="D16" s="476"/>
+      <c r="E16" s="476"/>
+      <c r="F16" s="476"/>
+      <c r="G16" s="476"/>
+      <c r="H16" s="476"/>
+      <c r="I16" s="476"/>
+      <c r="J16" s="476"/>
+      <c r="K16" s="476"/>
+      <c r="L16" s="476"/>
+      <c r="M16" s="476"/>
+      <c r="N16" s="479"/>
       <c r="Q16" s="413" t="s">
         <v>106</v>
       </c>
@@ -44032,64 +43966,64 @@
     </row>
     <row r="17" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A17" s="439"/>
-      <c r="B17" s="521" t="s">
+      <c r="B17" s="480" t="s">
         <v>104</v>
       </c>
-      <c r="C17" s="522"/>
-      <c r="D17" s="523"/>
-      <c r="E17" s="521" t="s">
+      <c r="C17" s="481"/>
+      <c r="D17" s="482"/>
+      <c r="E17" s="480" t="s">
         <v>102</v>
       </c>
-      <c r="F17" s="522"/>
-      <c r="G17" s="523"/>
-      <c r="H17" s="521" t="s">
+      <c r="F17" s="481"/>
+      <c r="G17" s="482"/>
+      <c r="H17" s="480" t="s">
         <v>103</v>
       </c>
-      <c r="I17" s="522"/>
-      <c r="J17" s="523"/>
-      <c r="K17" s="521" t="s">
+      <c r="I17" s="481"/>
+      <c r="J17" s="482"/>
+      <c r="K17" s="480" t="s">
         <v>72</v>
       </c>
-      <c r="L17" s="522"/>
-      <c r="M17" s="523"/>
+      <c r="L17" s="481"/>
+      <c r="M17" s="482"/>
       <c r="N17" s="440"/>
       <c r="Q17" s="414" t="s">
         <v>107</v>
       </c>
-      <c r="R17" s="412">
+      <c r="R17" s="412" t="e">
         <f>'Summer Weights'!AJ61</f>
-        <v>4.7496999999999998</v>
-      </c>
-      <c r="S17" s="408">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="S17" s="408" t="e">
         <f>'Summer Weights'!AE52</f>
-        <v>1.5595000000000001</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="T17" s="408"/>
-      <c r="U17" s="412">
+      <c r="U17" s="412" t="e">
         <f>'Summer Weights'!AK61</f>
-        <v>-0.38919999999999977</v>
-      </c>
-      <c r="V17" s="408">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V17" s="408" t="e">
         <f>'Summer Weights'!AF52</f>
-        <v>7.0016999999999996</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="W17" s="408"/>
-      <c r="X17" s="412">
+      <c r="X17" s="412" t="e">
         <f>'Summer Weights'!AL61</f>
-        <v>0.77072804517574856</v>
-      </c>
-      <c r="Y17" s="408">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y17" s="408" t="e">
         <f>'Summer Weights'!AG52</f>
-        <v>3.2029096365455167</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="Z17" s="408"/>
-      <c r="AA17" s="412">
+      <c r="AA17" s="412" t="e">
         <f>'Summer Weights'!AM61</f>
-        <v>4.7747439937281033E-2</v>
-      </c>
-      <c r="AB17" s="408">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB17" s="408" t="e">
         <f>'Summer Weights'!AH52</f>
-        <v>0.18703707902634226</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="AC17" s="408"/>
       <c r="AD17" s="405">
@@ -44850,45 +44784,45 @@
       <c r="N28" s="451"/>
     </row>
     <row r="29" spans="1:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="525" t="s">
+      <c r="A29" s="478" t="s">
         <v>100</v>
       </c>
-      <c r="B29" s="526"/>
-      <c r="C29" s="526"/>
-      <c r="D29" s="526"/>
-      <c r="E29" s="526"/>
-      <c r="F29" s="526"/>
-      <c r="G29" s="526"/>
-      <c r="H29" s="526"/>
-      <c r="I29" s="526"/>
-      <c r="J29" s="526"/>
-      <c r="K29" s="526"/>
-      <c r="L29" s="526"/>
-      <c r="M29" s="526"/>
-      <c r="N29" s="527"/>
+      <c r="B29" s="476"/>
+      <c r="C29" s="476"/>
+      <c r="D29" s="476"/>
+      <c r="E29" s="476"/>
+      <c r="F29" s="476"/>
+      <c r="G29" s="476"/>
+      <c r="H29" s="476"/>
+      <c r="I29" s="476"/>
+      <c r="J29" s="476"/>
+      <c r="K29" s="476"/>
+      <c r="L29" s="476"/>
+      <c r="M29" s="476"/>
+      <c r="N29" s="479"/>
     </row>
     <row r="30" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A30" s="439"/>
-      <c r="B30" s="521" t="s">
+      <c r="B30" s="480" t="s">
         <v>104</v>
       </c>
-      <c r="C30" s="522"/>
-      <c r="D30" s="523"/>
-      <c r="E30" s="521" t="s">
+      <c r="C30" s="481"/>
+      <c r="D30" s="482"/>
+      <c r="E30" s="480" t="s">
         <v>102</v>
       </c>
-      <c r="F30" s="522"/>
-      <c r="G30" s="523"/>
-      <c r="H30" s="521" t="s">
+      <c r="F30" s="481"/>
+      <c r="G30" s="482"/>
+      <c r="H30" s="480" t="s">
         <v>103</v>
       </c>
-      <c r="I30" s="522"/>
-      <c r="J30" s="523"/>
-      <c r="K30" s="521" t="s">
+      <c r="I30" s="481"/>
+      <c r="J30" s="482"/>
+      <c r="K30" s="480" t="s">
         <v>72</v>
       </c>
-      <c r="L30" s="522"/>
-      <c r="M30" s="523"/>
+      <c r="L30" s="481"/>
+      <c r="M30" s="482"/>
       <c r="N30" s="440"/>
     </row>
     <row r="31" spans="1:63" x14ac:dyDescent="0.25">
@@ -45958,15 +45892,15 @@
       </c>
       <c r="B59" s="86">
         <f>'Summer Weights'!AL46</f>
-        <v>5.1789754851130283</v>
+        <v>17.130122200684887</v>
       </c>
       <c r="C59" s="409">
         <f>'Summer Weights'!AN6</f>
-        <v>11.951146715571859</v>
-      </c>
-      <c r="D59" s="408">
+        <v>0</v>
+      </c>
+      <c r="D59" s="408" t="e">
         <f t="shared" si="27"/>
-        <v>0.43334548628417668</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="E59" s="405">
         <v>-0.32648441197031308</v>
@@ -46207,11 +46141,11 @@
         <v>-5.2460135362221633E-2</v>
       </c>
       <c r="N65" s="451"/>
-      <c r="W65" s="528" t="s">
+      <c r="W65" s="477" t="s">
         <v>139</v>
       </c>
-      <c r="X65" s="528"/>
-      <c r="Y65" s="528"/>
+      <c r="X65" s="477"/>
+      <c r="Y65" s="477"/>
       <c r="Z65" s="56"/>
       <c r="AA65" s="215" t="s">
         <v>131</v>
@@ -46489,11 +46423,11 @@
     </row>
     <row r="74" spans="1:41" x14ac:dyDescent="0.25">
       <c r="F74" s="454"/>
-      <c r="W74" s="528" t="s">
+      <c r="W74" s="477" t="s">
         <v>140</v>
       </c>
-      <c r="X74" s="528"/>
-      <c r="Y74" s="528"/>
+      <c r="X74" s="477"/>
+      <c r="Y74" s="477"/>
       <c r="Z74" s="56"/>
       <c r="AA74" s="56"/>
       <c r="AB74" s="56"/>
@@ -46575,24 +46509,24 @@
       <c r="X77" s="225">
         <v>4.8309999999999995</v>
       </c>
-      <c r="Y77" s="408">
+      <c r="Y77" s="408" t="e">
         <f>'Summer Weights'!AB52</f>
-        <v>10.304</v>
-      </c>
-      <c r="Z77" s="408">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z77" s="408" t="e">
         <f t="shared" si="30"/>
-        <v>0.46884704968944091</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="AA77" s="225">
         <v>5.1789754851130283</v>
       </c>
-      <c r="AB77" s="408">
+      <c r="AB77" s="408" t="e">
         <f>'Summer Weights'!AC52</f>
-        <v>11.951146715571859</v>
-      </c>
-      <c r="AC77" s="408">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC77" s="408" t="e">
         <f t="shared" si="31"/>
-        <v>0.43334548628417668</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="AD77" s="405">
         <v>-0.32648441197031308</v>
@@ -46911,23 +46845,6 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="R3:T3"/>
-    <mergeCell ref="U3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="AA3:AC3"/>
-    <mergeCell ref="Q2:AD2"/>
-    <mergeCell ref="W65:Y65"/>
-    <mergeCell ref="W74:Y74"/>
-    <mergeCell ref="Q13:AD13"/>
-    <mergeCell ref="R14:T14"/>
-    <mergeCell ref="U14:W14"/>
-    <mergeCell ref="X14:Z14"/>
-    <mergeCell ref="AA14:AC14"/>
-    <mergeCell ref="A29:N29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="H30:J30"/>
-    <mergeCell ref="K30:M30"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="E17:G17"/>
     <mergeCell ref="H17:J17"/>
@@ -46938,6 +46855,23 @@
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="K2:M2"/>
     <mergeCell ref="A16:N16"/>
+    <mergeCell ref="A29:N29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="H30:J30"/>
+    <mergeCell ref="K30:M30"/>
+    <mergeCell ref="W65:Y65"/>
+    <mergeCell ref="W74:Y74"/>
+    <mergeCell ref="Q13:AD13"/>
+    <mergeCell ref="R14:T14"/>
+    <mergeCell ref="U14:W14"/>
+    <mergeCell ref="X14:Z14"/>
+    <mergeCell ref="AA14:AC14"/>
+    <mergeCell ref="R3:T3"/>
+    <mergeCell ref="U3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="AA3:AC3"/>
+    <mergeCell ref="Q2:AD2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -51638,6 +51572,11 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="R1:S1"/>
+    <mergeCell ref="R14:S14"/>
+    <mergeCell ref="W1:X1"/>
+    <mergeCell ref="W14:X14"/>
+    <mergeCell ref="R56:S56"/>
     <mergeCell ref="R65:S65"/>
     <mergeCell ref="Y65:Z65"/>
     <mergeCell ref="R27:S27"/>
@@ -51648,11 +51587,6 @@
     <mergeCell ref="T65:U65"/>
     <mergeCell ref="T75:U75"/>
     <mergeCell ref="Y56:Z56"/>
-    <mergeCell ref="R1:S1"/>
-    <mergeCell ref="R14:S14"/>
-    <mergeCell ref="W1:X1"/>
-    <mergeCell ref="W14:X14"/>
-    <mergeCell ref="R56:S56"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>